<commit_message>
publish excel ko changed
</commit_message>
<xml_diff>
--- a/buda/mp4_publish_tracker.xlsx
+++ b/buda/mp4_publish_tracker.xlsx
@@ -4249,9 +4249,13 @@
         <v>1</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2025-06-07 04:55:22</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -4268,9 +4272,13 @@
         <v>1</v>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2025-06-07 10:55:22</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -4287,9 +4295,13 @@
         <v>1</v>
       </c>
       <c r="D17" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>2025-06-07 16:55:22</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -4306,9 +4318,13 @@
         <v>1</v>
       </c>
       <c r="D18" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2025-06-07 22:55:22</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -4325,9 +4341,13 @@
         <v>1</v>
       </c>
       <c r="D19" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2025-06-08 04:55:22</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -4344,9 +4364,13 @@
         <v>1</v>
       </c>
       <c r="D20" t="n">
-        <v>0</v>
-      </c>
-      <c r="E20" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>2025-06-08 10:55:22</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -4363,9 +4387,13 @@
         <v>1</v>
       </c>
       <c r="D21" t="n">
-        <v>0</v>
-      </c>
-      <c r="E21" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>2025-06-08 16:55:22</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -4382,9 +4410,13 @@
         <v>1</v>
       </c>
       <c r="D22" t="n">
-        <v>0</v>
-      </c>
-      <c r="E22" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>2025-06-08 22:55:22</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -4401,9 +4433,13 @@
         <v>1</v>
       </c>
       <c r="D23" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>2025-06-09 04:55:22</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -4420,9 +4456,13 @@
         <v>1</v>
       </c>
       <c r="D24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E24" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>2025-06-09 10:55:22</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -4439,9 +4479,13 @@
         <v>1</v>
       </c>
       <c r="D25" t="n">
-        <v>0</v>
-      </c>
-      <c r="E25" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>2025-06-09 16:55:22</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -4515,9 +4559,13 @@
         <v>1</v>
       </c>
       <c r="D29" t="n">
-        <v>0</v>
-      </c>
-      <c r="E29" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>2025-06-09 22:55:22</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -4534,9 +4582,13 @@
         <v>1</v>
       </c>
       <c r="D30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E30" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>2025-06-10 04:55:22</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">

</xml_diff>